<commit_message>
Added functionality to the Analyze Files to create a text file with all possible paths.  Also, fixed simulation_runner so it proper=ly handles inclusive paths.  Simulation is still not showing a different nmuber of completed tokens when the number of simulation days is incresed.
</commit_message>
<xml_diff>
--- a/5.5.13 Real Property-Monthly Reviews-Inclusive_results.xlsx
+++ b/5.5.13 Real Property-Monthly Reviews-Inclusive_results.xlsx
@@ -573,7 +573,7 @@
         <v>500</v>
       </c>
       <c r="D2" t="n">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="E2" t="n">
         <v>100</v>
@@ -582,31 +582,31 @@
         <v>36.79</v>
       </c>
       <c r="G2" t="n">
-        <v>58976</v>
+        <v>60439.95</v>
       </c>
       <c r="H2" t="n">
-        <v>35610.18</v>
+        <v>35095.94</v>
       </c>
       <c r="I2" t="n">
-        <v>41550.93</v>
+        <v>40436.66</v>
       </c>
       <c r="J2" t="n">
-        <v>15966.05</v>
+        <v>16001.12</v>
       </c>
       <c r="K2" t="n">
-        <v>53378.56</v>
+        <v>53468.09</v>
       </c>
       <c r="L2" t="n">
-        <v>6903549.88</v>
+        <v>6635918.64</v>
       </c>
       <c r="M2" t="n">
         <v>24.57</v>
       </c>
       <c r="N2" t="n">
-        <v>55056.17</v>
+        <v>60424.63</v>
       </c>
       <c r="O2" t="n">
-        <v>35402.82</v>
+        <v>34925.89</v>
       </c>
     </row>
     <row r="3">
@@ -687,19 +687,19 @@
         <v>9.58</v>
       </c>
       <c r="H4" t="n">
-        <v>8.09</v>
+        <v>8.039999999999999</v>
       </c>
       <c r="I4" t="n">
-        <v>8.34</v>
+        <v>8.25</v>
       </c>
       <c r="J4" t="n">
-        <v>1.1</v>
+        <v>1.11</v>
       </c>
       <c r="K4" t="n">
-        <v>9.380000000000001</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="L4" t="n">
-        <v>6644911.52</v>
+        <v>6644514.36</v>
       </c>
       <c r="M4" t="n">
         <v>5.92</v>
@@ -708,7 +708,7 @@
         <v>30167.53</v>
       </c>
       <c r="O4" t="n">
-        <v>13316.46</v>
+        <v>13315.66</v>
       </c>
     </row>
     <row r="5">
@@ -774,43 +774,43 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="D6" t="n">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="E6" t="n">
         <v>100</v>
       </c>
       <c r="F6" t="n">
-        <v>3.13</v>
+        <v>3.32</v>
       </c>
       <c r="G6" t="n">
-        <v>6.74</v>
+        <v>6.7</v>
       </c>
       <c r="H6" t="n">
-        <v>5.58</v>
+        <v>5.59</v>
       </c>
       <c r="I6" t="n">
-        <v>5.7</v>
+        <v>5.74</v>
       </c>
       <c r="J6" t="n">
-        <v>0.89</v>
+        <v>0.87</v>
       </c>
       <c r="K6" t="n">
-        <v>6.61</v>
+        <v>6.56</v>
       </c>
       <c r="L6" t="n">
-        <v>4996237.09</v>
+        <v>4752827.62</v>
       </c>
       <c r="M6" t="n">
         <v>24.57</v>
       </c>
       <c r="N6" t="n">
-        <v>45841.04</v>
+        <v>50345.07</v>
       </c>
       <c r="O6" t="n">
-        <v>31422.87</v>
+        <v>30862.52</v>
       </c>
     </row>
     <row r="7">
@@ -825,10 +825,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="D7" t="n">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="E7" t="n">
         <v>100</v>
@@ -876,43 +876,43 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="D8" t="n">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="E8" t="n">
         <v>100</v>
       </c>
       <c r="F8" t="n">
-        <v>73.98</v>
+        <v>70.16</v>
       </c>
       <c r="G8" t="n">
-        <v>162.31</v>
+        <v>163.29</v>
       </c>
       <c r="H8" t="n">
-        <v>130.27</v>
+        <v>129.8</v>
       </c>
       <c r="I8" t="n">
-        <v>139.72</v>
+        <v>132.23</v>
       </c>
       <c r="J8" t="n">
-        <v>24.78</v>
+        <v>24.33</v>
       </c>
       <c r="K8" t="n">
-        <v>160.07</v>
+        <v>159.39</v>
       </c>
       <c r="L8" t="n">
-        <v>1713885.45</v>
+        <v>1940412.23</v>
       </c>
       <c r="M8" t="n">
         <v>58.03</v>
       </c>
       <c r="N8" t="n">
-        <v>46037.06</v>
+        <v>50230.75</v>
       </c>
       <c r="O8" t="n">
-        <v>31738.62</v>
+        <v>32888.34</v>
       </c>
     </row>
     <row r="9">
@@ -927,10 +927,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="D9" t="n">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="E9" t="n">
         <v>100</v>
@@ -1029,31 +1029,31 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D11" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E11" t="n">
         <v>100</v>
       </c>
       <c r="F11" t="n">
-        <v>0.58</v>
+        <v>0.59</v>
       </c>
       <c r="G11" t="n">
-        <v>1.2</v>
+        <v>1.21</v>
       </c>
       <c r="H11" t="n">
-        <v>0.95</v>
+        <v>0.97</v>
       </c>
       <c r="I11" t="n">
-        <v>0.9399999999999999</v>
+        <v>1.09</v>
       </c>
       <c r="J11" t="n">
         <v>0.2</v>
       </c>
       <c r="K11" t="n">
-        <v>1.17</v>
+        <v>1.18</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
@@ -1079,7 +1079,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F196"/>
+  <dimension ref="A1:F191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1309,20 +1309,20 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Token-103</t>
+          <t>Token-9</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>45663.43333333333</v>
+        <v>45663.30277777778</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>45666.38277333997</v>
+        <v>45666.4043220333</v>
       </c>
       <c r="D10" t="n">
-        <v>4247.19</v>
+        <v>4466.22</v>
       </c>
       <c r="E10" t="n">
-        <v>4232.69</v>
+        <v>4451.63</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -1333,20 +1333,20 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Token-9</t>
+          <t>Token-10</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>45663.30277777778</v>
+        <v>45663.30416666667</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>45666.40681350995</v>
+        <v>45666.43068794462</v>
       </c>
       <c r="D11" t="n">
-        <v>4469.81</v>
+        <v>4502.19</v>
       </c>
       <c r="E11" t="n">
-        <v>4457.38</v>
+        <v>4487.45</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -1357,20 +1357,20 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Token-10</t>
+          <t>Token-11</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>45663.30416666667</v>
+        <v>45663.30555555555</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>45666.43275460203</v>
+        <v>45666.46025158058</v>
       </c>
       <c r="D12" t="n">
-        <v>4505.17</v>
+        <v>4542.76</v>
       </c>
       <c r="E12" t="n">
-        <v>4491.89</v>
+        <v>4527.87</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -1381,20 +1381,20 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Token-11</t>
+          <t>Token-12</t>
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>45663.30555555555</v>
+        <v>45663.30694444444</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>45666.46370625058</v>
+        <v>45666.48655165378</v>
       </c>
       <c r="D13" t="n">
-        <v>4547.74</v>
+        <v>4578.63</v>
       </c>
       <c r="E13" t="n">
-        <v>4533.83</v>
+        <v>4565.05</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -1405,20 +1405,20 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Token-12</t>
+          <t>Token-13</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>45663.30694444444</v>
+        <v>45663.30833333333</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>45666.48994302718</v>
+        <v>45666.50850656521</v>
       </c>
       <c r="D14" t="n">
-        <v>4583.52</v>
+        <v>4608.25</v>
       </c>
       <c r="E14" t="n">
-        <v>4572.42</v>
+        <v>4595.05</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -1429,20 +1429,20 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Token-13</t>
+          <t>Token-14</t>
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>45663.30833333333</v>
+        <v>45663.30972222222</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>45666.51155284017</v>
+        <v>45670.35142918802</v>
       </c>
       <c r="D15" t="n">
-        <v>4612.64</v>
+        <v>10140.06</v>
       </c>
       <c r="E15" t="n">
-        <v>4601.04</v>
+        <v>10126.59</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -1453,20 +1453,20 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Token-14</t>
+          <t>Token-15</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>45663.30972222222</v>
+        <v>45663.31111111111</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>45670.35835651266</v>
+        <v>45670.38118302629</v>
       </c>
       <c r="D16" t="n">
-        <v>10150.03</v>
+        <v>10180.9</v>
       </c>
       <c r="E16" t="n">
-        <v>10136.33</v>
+        <v>10168.12</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -1477,20 +1477,20 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Token-15</t>
+          <t>Token-16</t>
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>45663.31111111111</v>
+        <v>45663.3125</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>45670.39011883323</v>
+        <v>45670.40775234823</v>
       </c>
       <c r="D17" t="n">
-        <v>10193.77</v>
+        <v>10217.16</v>
       </c>
       <c r="E17" t="n">
-        <v>10180.33</v>
+        <v>10202.63</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -1501,20 +1501,20 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Token-16</t>
+          <t>Token-17</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>45663.3125</v>
+        <v>45663.31388888889</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>45670.41323506746</v>
+        <v>45670.42943357585</v>
       </c>
       <c r="D18" t="n">
-        <v>10225.06</v>
+        <v>10246.38</v>
       </c>
       <c r="E18" t="n">
-        <v>10211.95</v>
+        <v>10234.47</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -1525,24 +1525,24 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Token-17</t>
+          <t>Token-18</t>
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>45663.31388888889</v>
+        <v>45663.31527777778</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>45670.43331227839</v>
+        <v>45671.2924234587</v>
       </c>
       <c r="D19" t="n">
-        <v>10251.97</v>
+        <v>11487.09</v>
       </c>
       <c r="E19" t="n">
-        <v>10239.78</v>
+        <v>10295.37</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Inclusive Path 3 -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -1556,13 +1556,13 @@
         <v>45663.31666666667</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>45671.31823521901</v>
+        <v>45671.31847428666</v>
       </c>
       <c r="D20" t="n">
-        <v>11522.26</v>
+        <v>11522.6</v>
       </c>
       <c r="E20" t="n">
-        <v>11507.79</v>
+        <v>11508.13</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -1580,13 +1580,13 @@
         <v>45663.31805555556</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>45671.44603847308</v>
+        <v>45671.44627754073</v>
       </c>
       <c r="D21" t="n">
-        <v>11704.3</v>
+        <v>11704.64</v>
       </c>
       <c r="E21" t="n">
-        <v>11549.53</v>
+        <v>11549.88</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -1604,13 +1604,13 @@
         <v>45663.31944444445</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>45671.47168056735</v>
+        <v>45671.471919635</v>
       </c>
       <c r="D22" t="n">
-        <v>11739.22</v>
+        <v>11739.56</v>
       </c>
       <c r="E22" t="n">
-        <v>11724.9</v>
+        <v>11725.24</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -1628,13 +1628,13 @@
         <v>45663.32083333333</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>45671.49476474138</v>
+        <v>45671.49500380902</v>
       </c>
       <c r="D23" t="n">
-        <v>11770.46</v>
+        <v>11770.81</v>
       </c>
       <c r="E23" t="n">
-        <v>11757.59</v>
+        <v>11757.94</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -1652,13 +1652,13 @@
         <v>45663.32222222222</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>45671.51965701029</v>
+        <v>45671.51989607794</v>
       </c>
       <c r="D24" t="n">
-        <v>11804.31</v>
+        <v>11804.65</v>
       </c>
       <c r="E24" t="n">
-        <v>11791.17</v>
+        <v>11791.52</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -3253,44 +3253,44 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Token-95</t>
+          <t>Token-94</t>
         </is>
       </c>
       <c r="B91" s="2" t="n">
-        <v>45663.42222222222</v>
+        <v>45663.42083333333</v>
       </c>
       <c r="C91" s="2" t="n">
-        <v>45688.36367432446</v>
+        <v>45688.36095416668</v>
       </c>
       <c r="D91" t="n">
-        <v>35915.69</v>
+        <v>35913.77</v>
       </c>
       <c r="E91" t="n">
-        <v>35901.87</v>
+        <v>35806.26</v>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Inclusive Path 3 -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Token-97</t>
+          <t>Token-95</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
-        <v>45663.425</v>
+        <v>45663.42222222222</v>
       </c>
       <c r="C92" s="2" t="n">
-        <v>45688.46745742904</v>
+        <v>45688.36367432446</v>
       </c>
       <c r="D92" t="n">
-        <v>36061.14</v>
+        <v>35915.69</v>
       </c>
       <c r="E92" t="n">
-        <v>36046.1</v>
+        <v>35901.87</v>
       </c>
       <c r="F92" t="inlineStr">
         <is>
@@ -3301,116 +3301,116 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Token-98</t>
+          <t>Token-96</t>
         </is>
       </c>
       <c r="B93" s="2" t="n">
-        <v>45663.42638888889</v>
+        <v>45663.42361111111</v>
       </c>
       <c r="C93" s="2" t="n">
-        <v>45688.47136238746</v>
+        <v>45688.43577673551</v>
       </c>
       <c r="D93" t="n">
-        <v>36064.76</v>
+        <v>36017.52</v>
       </c>
       <c r="E93" t="n">
-        <v>36050.51</v>
+        <v>35904.99</v>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Inclusive Path 3 -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Token-99</t>
+          <t>Token-97</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
-        <v>45663.42777777778</v>
+        <v>45663.425</v>
       </c>
       <c r="C94" s="2" t="n">
-        <v>45691.29248321267</v>
+        <v>45688.43945211066</v>
       </c>
       <c r="D94" t="n">
-        <v>40125.18</v>
+        <v>36020.81</v>
       </c>
       <c r="E94" t="n">
-        <v>36054.76</v>
+        <v>36006.5</v>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Inclusive Path 3 -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Token-100</t>
+          <t>Token-98</t>
         </is>
       </c>
       <c r="B95" s="2" t="n">
-        <v>45663.42916666667</v>
+        <v>45663.42638888889</v>
       </c>
       <c r="C95" s="2" t="n">
-        <v>45691.37888401765</v>
+        <v>45688.44291673348</v>
       </c>
       <c r="D95" t="n">
-        <v>40247.59</v>
+        <v>36023.8</v>
       </c>
       <c r="E95" t="n">
-        <v>40115.44</v>
+        <v>36010.18</v>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Inclusive Path 3 -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Token-102</t>
+          <t>Token-99</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
-        <v>45663.43194444444</v>
+        <v>45663.42777777778</v>
       </c>
       <c r="C96" s="2" t="n">
-        <v>45691.49452945108</v>
+        <v>45691.2924352856</v>
       </c>
       <c r="D96" t="n">
-        <v>40410.12</v>
+        <v>40125.11</v>
       </c>
       <c r="E96" t="n">
-        <v>40396.03</v>
+        <v>36013.8</v>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Inclusive Path 3 -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Token-104</t>
+          <t>Token-102</t>
         </is>
       </c>
       <c r="B97" s="2" t="n">
-        <v>45663.43472222222</v>
+        <v>45663.43194444444</v>
       </c>
       <c r="C97" s="2" t="n">
-        <v>45691.49768049315</v>
+        <v>45691.51295620496</v>
       </c>
       <c r="D97" t="n">
-        <v>40410.66</v>
+        <v>40436.66</v>
       </c>
       <c r="E97" t="n">
-        <v>40399.13</v>
+        <v>40422.74</v>
       </c>
       <c r="F97" t="inlineStr">
         <is>
@@ -3421,20 +3421,20 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Token-105</t>
+          <t>Token-103</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
-        <v>45663.43611111111</v>
+        <v>45663.43333333333</v>
       </c>
       <c r="C98" s="2" t="n">
-        <v>45691.50035067376</v>
+        <v>45691.51617941971</v>
       </c>
       <c r="D98" t="n">
-        <v>40412.5</v>
+        <v>40439.3</v>
       </c>
       <c r="E98" t="n">
-        <v>40400</v>
+        <v>40425.24</v>
       </c>
       <c r="F98" t="inlineStr">
         <is>
@@ -3445,44 +3445,44 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Token-106</t>
+          <t>Token-104</t>
         </is>
       </c>
       <c r="B99" s="2" t="n">
-        <v>45663.4375</v>
+        <v>45663.43472222222</v>
       </c>
       <c r="C99" s="2" t="n">
-        <v>45692.29230932343</v>
+        <v>45691.5203095691</v>
       </c>
       <c r="D99" t="n">
-        <v>41550.93</v>
+        <v>40443.25</v>
       </c>
       <c r="E99" t="n">
-        <v>40404.44</v>
+        <v>40429.93</v>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Inclusive Path 3 -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Token-107</t>
+          <t>Token-105</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
-        <v>45663.43888888889</v>
+        <v>45663.43611111111</v>
       </c>
       <c r="C100" s="2" t="n">
-        <v>45692.29492207238</v>
+        <v>45691.52387611951</v>
       </c>
       <c r="D100" t="n">
-        <v>41552.69</v>
+        <v>40446.38</v>
       </c>
       <c r="E100" t="n">
-        <v>41539.55</v>
+        <v>40434.26</v>
       </c>
       <c r="F100" t="inlineStr">
         <is>
@@ -3493,20 +3493,20 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Token-108</t>
+          <t>Token-106</t>
         </is>
       </c>
       <c r="B101" s="2" t="n">
-        <v>45663.44027777778</v>
+        <v>45663.4375</v>
       </c>
       <c r="C101" s="2" t="n">
-        <v>45692.29928341222</v>
+        <v>45691.52791131251</v>
       </c>
       <c r="D101" t="n">
-        <v>41556.97</v>
+        <v>40450.19</v>
       </c>
       <c r="E101" t="n">
-        <v>41542.97</v>
+        <v>40437.74</v>
       </c>
       <c r="F101" t="inlineStr">
         <is>
@@ -3517,20 +3517,20 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Token-109</t>
+          <t>Token-107</t>
         </is>
       </c>
       <c r="B102" s="2" t="n">
-        <v>45663.44166666667</v>
+        <v>45663.43888888889</v>
       </c>
       <c r="C102" s="2" t="n">
-        <v>45692.30396307021</v>
+        <v>45691.53242491442</v>
       </c>
       <c r="D102" t="n">
-        <v>41561.71</v>
+        <v>40454.69</v>
       </c>
       <c r="E102" t="n">
-        <v>41546.86</v>
+        <v>40439.69</v>
       </c>
       <c r="F102" t="inlineStr">
         <is>
@@ -3541,20 +3541,20 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Token-111</t>
+          <t>Token-108</t>
         </is>
       </c>
       <c r="B103" s="2" t="n">
-        <v>45663.44444444445</v>
+        <v>45663.44027777778</v>
       </c>
       <c r="C103" s="2" t="n">
-        <v>45692.41747330894</v>
+        <v>45691.53695006271</v>
       </c>
       <c r="D103" t="n">
-        <v>41721.16</v>
+        <v>40459.21</v>
       </c>
       <c r="E103" t="n">
-        <v>41710.1</v>
+        <v>40444.22</v>
       </c>
       <c r="F103" t="inlineStr">
         <is>
@@ -3565,20 +3565,20 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Token-112</t>
+          <t>Token-110</t>
         </is>
       </c>
       <c r="B104" s="2" t="n">
-        <v>45663.44583333333</v>
+        <v>45663.44305555556</v>
       </c>
       <c r="C104" s="2" t="n">
-        <v>45692.42191308398</v>
+        <v>45692.29575701972</v>
       </c>
       <c r="D104" t="n">
-        <v>41725.55</v>
+        <v>41547.89</v>
       </c>
       <c r="E104" t="n">
-        <v>41712.94</v>
+        <v>41534.23</v>
       </c>
       <c r="F104" t="inlineStr">
         <is>
@@ -3589,20 +3589,20 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Token-113</t>
+          <t>Token-111</t>
         </is>
       </c>
       <c r="B105" s="2" t="n">
-        <v>45663.44722222222</v>
+        <v>45663.44444444445</v>
       </c>
       <c r="C105" s="2" t="n">
-        <v>45692.42609832081</v>
+        <v>45692.30010264531</v>
       </c>
       <c r="D105" t="n">
-        <v>41729.58</v>
+        <v>41552.15</v>
       </c>
       <c r="E105" t="n">
-        <v>41715.11</v>
+        <v>41538.57</v>
       </c>
       <c r="F105" t="inlineStr">
         <is>
@@ -3613,20 +3613,20 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Token-114</t>
+          <t>Token-112</t>
         </is>
       </c>
       <c r="B106" s="2" t="n">
-        <v>45663.44861111111</v>
+        <v>45663.44583333333</v>
       </c>
       <c r="C106" s="2" t="n">
-        <v>45692.43058071769</v>
+        <v>45692.30374908002</v>
       </c>
       <c r="D106" t="n">
-        <v>41734.04</v>
+        <v>41555.4</v>
       </c>
       <c r="E106" t="n">
-        <v>41719.21</v>
+        <v>41543.94</v>
       </c>
       <c r="F106" t="inlineStr">
         <is>
@@ -3637,44 +3637,44 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Token-115</t>
+          <t>Token-113</t>
         </is>
       </c>
       <c r="B107" s="2" t="n">
-        <v>45663.45</v>
+        <v>45663.44722222222</v>
       </c>
       <c r="C107" s="2" t="n">
-        <v>45692.52851028481</v>
+        <v>45692.30792187</v>
       </c>
       <c r="D107" t="n">
-        <v>41873.05</v>
+        <v>41559.41</v>
       </c>
       <c r="E107" t="n">
-        <v>41723.42</v>
+        <v>41547.18</v>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Inclusive Path 3 -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Token-116</t>
+          <t>Token-114</t>
         </is>
       </c>
       <c r="B108" s="2" t="n">
-        <v>45663.45138888889</v>
+        <v>45663.44861111111</v>
       </c>
       <c r="C108" s="2" t="n">
-        <v>45692.53181303672</v>
+        <v>45692.31114815334</v>
       </c>
       <c r="D108" t="n">
-        <v>41875.81</v>
+        <v>41562.05</v>
       </c>
       <c r="E108" t="n">
-        <v>41862.68</v>
+        <v>41549.36</v>
       </c>
       <c r="F108" t="inlineStr">
         <is>
@@ -3685,20 +3685,20 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Token-117</t>
+          <t>Token-115</t>
         </is>
       </c>
       <c r="B109" s="2" t="n">
-        <v>45663.45277777778</v>
+        <v>45663.45</v>
       </c>
       <c r="C109" s="2" t="n">
-        <v>45692.53587500706</v>
+        <v>45692.31515831483</v>
       </c>
       <c r="D109" t="n">
-        <v>41879.66</v>
+        <v>41565.83</v>
       </c>
       <c r="E109" t="n">
-        <v>41865.68</v>
+        <v>41552.82</v>
       </c>
       <c r="F109" t="inlineStr">
         <is>
@@ -3709,20 +3709,20 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Token-118</t>
+          <t>Token-116</t>
         </is>
       </c>
       <c r="B110" s="2" t="n">
-        <v>45663.45416666667</v>
+        <v>45663.45138888889</v>
       </c>
       <c r="C110" s="2" t="n">
-        <v>45692.53936202844</v>
+        <v>45692.31952693585</v>
       </c>
       <c r="D110" t="n">
-        <v>41882.68</v>
+        <v>41570.12</v>
       </c>
       <c r="E110" t="n">
-        <v>41868.84</v>
+        <v>41555.41</v>
       </c>
       <c r="F110" t="inlineStr">
         <is>
@@ -3733,20 +3733,20 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Token-119</t>
+          <t>Token-117</t>
         </is>
       </c>
       <c r="B111" s="2" t="n">
-        <v>45663.45555555556</v>
+        <v>45663.45277777778</v>
       </c>
       <c r="C111" s="2" t="n">
-        <v>45693.29166666666</v>
+        <v>45692.3234546303</v>
       </c>
       <c r="D111" t="n">
-        <v>42964</v>
+        <v>41573.77</v>
       </c>
       <c r="E111" t="n">
-        <v>41872.51</v>
+        <v>41559.23</v>
       </c>
       <c r="F111" t="inlineStr">
         <is>
@@ -3757,20 +3757,20 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Token-120</t>
+          <t>Token-118</t>
         </is>
       </c>
       <c r="B112" s="2" t="n">
-        <v>45663.45694444444</v>
+        <v>45663.45416666667</v>
       </c>
       <c r="C112" s="2" t="n">
-        <v>45693.29633249367</v>
+        <v>45692.3274410761</v>
       </c>
       <c r="D112" t="n">
-        <v>42968.72</v>
+        <v>41577.52</v>
       </c>
       <c r="E112" t="n">
-        <v>42952.47</v>
+        <v>41563.64</v>
       </c>
       <c r="F112" t="inlineStr">
         <is>
@@ -3781,92 +3781,92 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Token-121</t>
+          <t>Token-120</t>
         </is>
       </c>
       <c r="B113" s="2" t="n">
-        <v>45663.45833333334</v>
+        <v>45663.45694444444</v>
       </c>
       <c r="C113" s="2" t="n">
-        <v>45693.36223602526</v>
+        <v>45692.40369051745</v>
       </c>
       <c r="D113" t="n">
-        <v>43061.62</v>
+        <v>41683.31</v>
       </c>
       <c r="E113" t="n">
-        <v>42958.22</v>
+        <v>41669.44</v>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Inclusive Path 3 -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Token-122</t>
+          <t>Token-121</t>
         </is>
       </c>
       <c r="B114" s="2" t="n">
-        <v>45663.45972222222</v>
+        <v>45663.45833333334</v>
       </c>
       <c r="C114" s="2" t="n">
-        <v>45693.46894948309</v>
+        <v>45692.40830754777</v>
       </c>
       <c r="D114" t="n">
-        <v>43213.29</v>
+        <v>41687.96</v>
       </c>
       <c r="E114" t="n">
-        <v>43049.77</v>
+        <v>41674.01</v>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Inclusive Path 3 -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Token-123</t>
+          <t>Token-122</t>
         </is>
       </c>
       <c r="B115" s="2" t="n">
-        <v>45663.46111111111</v>
+        <v>45663.45972222222</v>
       </c>
       <c r="C115" s="2" t="n">
-        <v>45693.4719571422</v>
+        <v>45692.52234586569</v>
       </c>
       <c r="D115" t="n">
-        <v>43215.62</v>
+        <v>41850.18</v>
       </c>
       <c r="E115" t="n">
-        <v>43201.56</v>
+        <v>41677.47</v>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Inclusive Path 3 -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Token-124</t>
+          <t>Token-123</t>
         </is>
       </c>
       <c r="B116" s="2" t="n">
-        <v>45663.4625</v>
+        <v>45663.46111111111</v>
       </c>
       <c r="C116" s="2" t="n">
-        <v>45693.47613081274</v>
+        <v>45692.52462880291</v>
       </c>
       <c r="D116" t="n">
-        <v>43219.63</v>
+        <v>41851.47</v>
       </c>
       <c r="E116" t="n">
-        <v>43204.84</v>
+        <v>41837.82</v>
       </c>
       <c r="F116" t="inlineStr">
         <is>
@@ -3877,20 +3877,20 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Token-125</t>
+          <t>Token-124</t>
         </is>
       </c>
       <c r="B117" s="2" t="n">
-        <v>45663.46388888889</v>
+        <v>45663.4625</v>
       </c>
       <c r="C117" s="2" t="n">
-        <v>45693.48021012398</v>
+        <v>45692.52915281743</v>
       </c>
       <c r="D117" t="n">
-        <v>43223.5</v>
+        <v>41855.98</v>
       </c>
       <c r="E117" t="n">
-        <v>43211.14</v>
+        <v>41841.44</v>
       </c>
       <c r="F117" t="inlineStr">
         <is>
@@ -3901,20 +3901,20 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Token-126</t>
+          <t>Token-125</t>
         </is>
       </c>
       <c r="B118" s="2" t="n">
-        <v>45663.46527777778</v>
+        <v>45663.46388888889</v>
       </c>
       <c r="C118" s="2" t="n">
-        <v>45693.48337377871</v>
+        <v>45692.53256641854</v>
       </c>
       <c r="D118" t="n">
-        <v>43226.06</v>
+        <v>41858.9</v>
       </c>
       <c r="E118" t="n">
-        <v>43215.01</v>
+        <v>41845.2</v>
       </c>
       <c r="F118" t="inlineStr">
         <is>
@@ -3925,24 +3925,24 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Token-127</t>
+          <t>Token-126</t>
         </is>
       </c>
       <c r="B119" s="2" t="n">
-        <v>45663.46666666667</v>
+        <v>45663.46527777778</v>
       </c>
       <c r="C119" s="2" t="n">
-        <v>45694.2922687041</v>
+        <v>45692.53711632572</v>
       </c>
       <c r="D119" t="n">
-        <v>44388.87</v>
+        <v>41863.45</v>
       </c>
       <c r="E119" t="n">
-        <v>43216.84</v>
+        <v>41850.35</v>
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Inclusive Path 3 -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -3956,17 +3956,17 @@
         <v>45663.46805555555</v>
       </c>
       <c r="C120" s="2" t="n">
-        <v>45694.29628764397</v>
+        <v>45693.36765631063</v>
       </c>
       <c r="D120" t="n">
-        <v>44392.65</v>
+        <v>43055.43</v>
       </c>
       <c r="E120" t="n">
-        <v>44376.99</v>
+        <v>42937.62</v>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Inclusive Path 3 -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -3980,13 +3980,13 @@
         <v>45663.46944444445</v>
       </c>
       <c r="C121" s="2" t="n">
-        <v>45694.30007855481</v>
+        <v>45693.37004207973</v>
       </c>
       <c r="D121" t="n">
-        <v>44396.11</v>
+        <v>43056.86</v>
       </c>
       <c r="E121" t="n">
-        <v>43305.28</v>
+        <v>41963.61</v>
       </c>
       <c r="F121" t="inlineStr">
         <is>
@@ -4004,37 +4004,37 @@
         <v>45663.47083333333</v>
       </c>
       <c r="C122" s="2" t="n">
-        <v>45694.38574429815</v>
+        <v>45693.37248898116</v>
       </c>
       <c r="D122" t="n">
-        <v>44517.47</v>
+        <v>43058.38</v>
       </c>
       <c r="E122" t="n">
-        <v>44386.66</v>
+        <v>43046.61</v>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Inclusive Path 3 -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Token-131</t>
+          <t>Token-132</t>
         </is>
       </c>
       <c r="B123" s="2" t="n">
-        <v>45663.47222222222</v>
+        <v>45663.47361111111</v>
       </c>
       <c r="C123" s="2" t="n">
-        <v>45694.38910878559</v>
+        <v>45693.45539659362</v>
       </c>
       <c r="D123" t="n">
-        <v>44520.32</v>
+        <v>43173.77</v>
       </c>
       <c r="E123" t="n">
-        <v>44505.91</v>
+        <v>43158.96</v>
       </c>
       <c r="F123" t="inlineStr">
         <is>
@@ -4045,20 +4045,20 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Token-132</t>
+          <t>Token-133</t>
         </is>
       </c>
       <c r="B124" s="2" t="n">
-        <v>45663.47361111111</v>
+        <v>45663.475</v>
       </c>
       <c r="C124" s="2" t="n">
-        <v>45694.39249420038</v>
+        <v>45693.45934744553</v>
       </c>
       <c r="D124" t="n">
-        <v>44523.19</v>
+        <v>43177.46</v>
       </c>
       <c r="E124" t="n">
-        <v>44508.79</v>
+        <v>43162.88</v>
       </c>
       <c r="F124" t="inlineStr">
         <is>
@@ -4069,20 +4069,20 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Token-133</t>
+          <t>Token-134</t>
         </is>
       </c>
       <c r="B125" s="2" t="n">
-        <v>45663.475</v>
+        <v>45663.47638888889</v>
       </c>
       <c r="C125" s="2" t="n">
-        <v>45694.39714030011</v>
+        <v>45693.46392779545</v>
       </c>
       <c r="D125" t="n">
-        <v>44527.88</v>
+        <v>43182.06</v>
       </c>
       <c r="E125" t="n">
-        <v>44514.59</v>
+        <v>43167.89</v>
       </c>
       <c r="F125" t="inlineStr">
         <is>
@@ -4093,20 +4093,20 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Token-134</t>
+          <t>Token-135</t>
         </is>
       </c>
       <c r="B126" s="2" t="n">
-        <v>45663.47638888889</v>
+        <v>45663.47777777778</v>
       </c>
       <c r="C126" s="2" t="n">
-        <v>45694.40151471234</v>
+        <v>45693.46793546191</v>
       </c>
       <c r="D126" t="n">
-        <v>44532.18</v>
+        <v>43185.83</v>
       </c>
       <c r="E126" t="n">
-        <v>44518.2</v>
+        <v>43171.9</v>
       </c>
       <c r="F126" t="inlineStr">
         <is>
@@ -4117,44 +4117,44 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Token-135</t>
+          <t>Token-136</t>
         </is>
       </c>
       <c r="B127" s="2" t="n">
-        <v>45663.47777777778</v>
+        <v>45663.47916666666</v>
       </c>
       <c r="C127" s="2" t="n">
-        <v>45694.40419965419</v>
+        <v>45694.29244972762</v>
       </c>
       <c r="D127" t="n">
-        <v>44534.05</v>
+        <v>44371.13</v>
       </c>
       <c r="E127" t="n">
-        <v>44522.11</v>
+        <v>43175.29</v>
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Inclusive Path 3 -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Token-136</t>
+          <t>Token-137</t>
         </is>
       </c>
       <c r="B128" s="2" t="n">
-        <v>45663.47916666666</v>
+        <v>45663.48055555556</v>
       </c>
       <c r="C128" s="2" t="n">
-        <v>45694.40841282097</v>
+        <v>45694.29494805498</v>
       </c>
       <c r="D128" t="n">
-        <v>44538.11</v>
+        <v>44372.73</v>
       </c>
       <c r="E128" t="n">
-        <v>44523.88</v>
+        <v>44361.32</v>
       </c>
       <c r="F128" t="inlineStr">
         <is>
@@ -4165,20 +4165,20 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Token-137</t>
+          <t>Token-138</t>
         </is>
       </c>
       <c r="B129" s="2" t="n">
-        <v>45663.48055555556</v>
+        <v>45663.48194444444</v>
       </c>
       <c r="C129" s="2" t="n">
-        <v>45694.41299134515</v>
+        <v>45694.29820884159</v>
       </c>
       <c r="D129" t="n">
-        <v>44542.71</v>
+        <v>44375.42</v>
       </c>
       <c r="E129" t="n">
-        <v>44526.87</v>
+        <v>44363.24</v>
       </c>
       <c r="F129" t="inlineStr">
         <is>
@@ -4189,44 +4189,44 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Token-138</t>
+          <t>Token-140</t>
         </is>
       </c>
       <c r="B130" s="2" t="n">
-        <v>45663.48194444444</v>
+        <v>45663.48472222222</v>
       </c>
       <c r="C130" s="2" t="n">
-        <v>45694.41557318978</v>
+        <v>45694.4813139835</v>
       </c>
       <c r="D130" t="n">
-        <v>44544.43</v>
+        <v>44635.09</v>
       </c>
       <c r="E130" t="n">
-        <v>44533.77</v>
+        <v>44525.14</v>
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Inclusive Path 3 -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Token-139</t>
+          <t>Token-141</t>
         </is>
       </c>
       <c r="B131" s="2" t="n">
-        <v>45663.48333333333</v>
+        <v>45663.48611111111</v>
       </c>
       <c r="C131" s="2" t="n">
-        <v>45694.41859381723</v>
+        <v>45694.48482202543</v>
       </c>
       <c r="D131" t="n">
-        <v>44546.78</v>
+        <v>44638.14</v>
       </c>
       <c r="E131" t="n">
-        <v>44535.94</v>
+        <v>44622.94</v>
       </c>
       <c r="F131" t="inlineStr">
         <is>
@@ -4237,20 +4237,20 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Token-141</t>
+          <t>Token-142</t>
         </is>
       </c>
       <c r="B132" s="2" t="n">
-        <v>45663.48611111111</v>
+        <v>45663.4875</v>
       </c>
       <c r="C132" s="2" t="n">
-        <v>45694.5123449561</v>
+        <v>45694.48712668361</v>
       </c>
       <c r="D132" t="n">
-        <v>44677.78</v>
+        <v>44639.46</v>
       </c>
       <c r="E132" t="n">
-        <v>44663.95</v>
+        <v>44626.68</v>
       </c>
       <c r="F132" t="inlineStr">
         <is>
@@ -4261,20 +4261,20 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Token-142</t>
+          <t>Token-143</t>
         </is>
       </c>
       <c r="B133" s="2" t="n">
-        <v>45663.4875</v>
+        <v>45663.48888888889</v>
       </c>
       <c r="C133" s="2" t="n">
-        <v>45694.51672394622</v>
+        <v>45694.49047233121</v>
       </c>
       <c r="D133" t="n">
-        <v>44682.08</v>
+        <v>44642.28</v>
       </c>
       <c r="E133" t="n">
-        <v>44668.26</v>
+        <v>44629.6</v>
       </c>
       <c r="F133" t="inlineStr">
         <is>
@@ -4285,20 +4285,20 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Token-143</t>
+          <t>Token-144</t>
         </is>
       </c>
       <c r="B134" s="2" t="n">
-        <v>45663.48888888889</v>
+        <v>45663.49027777778</v>
       </c>
       <c r="C134" s="2" t="n">
-        <v>45694.51988677818</v>
+        <v>45694.49454063218</v>
       </c>
       <c r="D134" t="n">
-        <v>44684.64</v>
+        <v>44646.14</v>
       </c>
       <c r="E134" t="n">
-        <v>44673.21</v>
+        <v>44632.47</v>
       </c>
       <c r="F134" t="inlineStr">
         <is>
@@ -4316,13 +4316,13 @@
         <v>45663.49166666667</v>
       </c>
       <c r="C135" s="2" t="n">
-        <v>45695.29626335535</v>
+        <v>45694.49879111957</v>
       </c>
       <c r="D135" t="n">
-        <v>45798.62</v>
+        <v>44650.26</v>
       </c>
       <c r="E135" t="n">
-        <v>45783.98</v>
+        <v>44638.7</v>
       </c>
       <c r="F135" t="inlineStr">
         <is>
@@ -4340,13 +4340,13 @@
         <v>45663.49305555555</v>
       </c>
       <c r="C136" s="2" t="n">
-        <v>45695.30051384274</v>
+        <v>45694.50331555337</v>
       </c>
       <c r="D136" t="n">
-        <v>45802.74</v>
+        <v>44654.77</v>
       </c>
       <c r="E136" t="n">
-        <v>45788.05</v>
+        <v>44638.95</v>
       </c>
       <c r="F136" t="inlineStr">
         <is>
@@ -4364,61 +4364,61 @@
         <v>45663.49444444444</v>
       </c>
       <c r="C137" s="2" t="n">
-        <v>45695.30503827654</v>
+        <v>45695.29225640342</v>
       </c>
       <c r="D137" t="n">
-        <v>45807.26</v>
+        <v>45788.85</v>
       </c>
       <c r="E137" t="n">
-        <v>45792.08</v>
+        <v>44644.13</v>
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Inclusive Path 3 -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Token-148</t>
+          <t>Token-149</t>
         </is>
       </c>
       <c r="B138" s="2" t="n">
-        <v>45663.49583333333</v>
+        <v>45663.49722222222</v>
       </c>
       <c r="C138" s="2" t="n">
-        <v>45695.39321155041</v>
+        <v>45695.3796660912</v>
       </c>
       <c r="D138" t="n">
-        <v>45932.22</v>
+        <v>45910.72</v>
       </c>
       <c r="E138" t="n">
-        <v>45795.84</v>
+        <v>45897.94</v>
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Inclusive Path 3 -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Token-149</t>
+          <t>Token-150</t>
         </is>
       </c>
       <c r="B139" s="2" t="n">
-        <v>45663.49722222222</v>
+        <v>45663.49861111111</v>
       </c>
       <c r="C139" s="2" t="n">
-        <v>45695.39626633422</v>
+        <v>45695.3821066985</v>
       </c>
       <c r="D139" t="n">
-        <v>45934.62</v>
+        <v>45912.23</v>
       </c>
       <c r="E139" t="n">
-        <v>45919.86</v>
+        <v>45899.69</v>
       </c>
       <c r="F139" t="inlineStr">
         <is>
@@ -4429,20 +4429,20 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Token-150</t>
+          <t>Token-151</t>
         </is>
       </c>
       <c r="B140" s="2" t="n">
-        <v>45663.49861111111</v>
+        <v>45663.5</v>
       </c>
       <c r="C140" s="2" t="n">
-        <v>45695.39923773643</v>
+        <v>45695.38504658671</v>
       </c>
       <c r="D140" t="n">
-        <v>45936.9</v>
+        <v>45914.47</v>
       </c>
       <c r="E140" t="n">
-        <v>45924.7</v>
+        <v>45901.71</v>
       </c>
       <c r="F140" t="inlineStr">
         <is>
@@ -4453,20 +4453,20 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Token-151</t>
+          <t>Token-152</t>
         </is>
       </c>
       <c r="B141" s="2" t="n">
-        <v>45663.5</v>
+        <v>45663.50138888889</v>
       </c>
       <c r="C141" s="2" t="n">
-        <v>45695.40391746548</v>
+        <v>45695.38770220346</v>
       </c>
       <c r="D141" t="n">
-        <v>45941.64</v>
+        <v>45916.29</v>
       </c>
       <c r="E141" t="n">
-        <v>45926.36</v>
+        <v>45904.28</v>
       </c>
       <c r="F141" t="inlineStr">
         <is>
@@ -4477,44 +4477,44 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>Token-152</t>
+          <t>Token-153</t>
         </is>
       </c>
       <c r="B142" s="2" t="n">
-        <v>45663.50138888889</v>
+        <v>45663.50277777778</v>
       </c>
       <c r="C142" s="2" t="n">
-        <v>45695.50484410077</v>
+        <v>45695.39229595376</v>
       </c>
       <c r="D142" t="n">
-        <v>46084.98</v>
+        <v>45920.91</v>
       </c>
       <c r="E142" t="n">
-        <v>45932.41</v>
+        <v>45905.92</v>
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Inclusive Path 3 -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Token-153</t>
+          <t>Token-155</t>
         </is>
       </c>
       <c r="B143" s="2" t="n">
-        <v>45663.50277777778</v>
+        <v>45663.50555555556</v>
       </c>
       <c r="C143" s="2" t="n">
-        <v>45695.50865917094</v>
+        <v>45695.50448993844</v>
       </c>
       <c r="D143" t="n">
-        <v>46088.47</v>
+        <v>46078.47</v>
       </c>
       <c r="E143" t="n">
-        <v>46074.57</v>
+        <v>46063.74</v>
       </c>
       <c r="F143" t="inlineStr">
         <is>
@@ -4525,44 +4525,44 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>Token-154</t>
+          <t>Token-156</t>
         </is>
       </c>
       <c r="B144" s="2" t="n">
-        <v>45663.50416666667</v>
+        <v>45663.50694444445</v>
       </c>
       <c r="C144" s="2" t="n">
-        <v>45698.29237551587</v>
+        <v>45695.50727075987</v>
       </c>
       <c r="D144" t="n">
-        <v>50095.02</v>
+        <v>46080.47</v>
       </c>
       <c r="E144" t="n">
-        <v>46080.6</v>
+        <v>46067.37</v>
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Inclusive Path 3 -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Token-155</t>
+          <t>Token-157</t>
         </is>
       </c>
       <c r="B145" s="2" t="n">
-        <v>45663.50555555556</v>
+        <v>45663.50833333333</v>
       </c>
       <c r="C145" s="2" t="n">
-        <v>45698.29613261452</v>
+        <v>45695.51086182544</v>
       </c>
       <c r="D145" t="n">
-        <v>50098.43</v>
+        <v>46083.64</v>
       </c>
       <c r="E145" t="n">
-        <v>50082.5</v>
+        <v>46071.4</v>
       </c>
       <c r="F145" t="inlineStr">
         <is>
@@ -4573,20 +4573,20 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Token-156</t>
+          <t>Token-158</t>
         </is>
       </c>
       <c r="B146" s="2" t="n">
-        <v>45663.50694444445</v>
+        <v>45663.50972222222</v>
       </c>
       <c r="C146" s="2" t="n">
-        <v>45698.29891343596</v>
+        <v>45695.5147155672</v>
       </c>
       <c r="D146" t="n">
-        <v>50100.44</v>
+        <v>46087.19</v>
       </c>
       <c r="E146" t="n">
-        <v>50090.91</v>
+        <v>46075.38</v>
       </c>
       <c r="F146" t="inlineStr">
         <is>
@@ -4597,20 +4597,20 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Token-157</t>
+          <t>Token-159</t>
         </is>
       </c>
       <c r="B147" s="2" t="n">
-        <v>45663.50833333333</v>
+        <v>45663.51111111111</v>
       </c>
       <c r="C147" s="2" t="n">
-        <v>45698.30250450153</v>
+        <v>45695.51818366436</v>
       </c>
       <c r="D147" t="n">
-        <v>50103.61</v>
+        <v>46090.18</v>
       </c>
       <c r="E147" t="n">
-        <v>50091.17</v>
+        <v>46079.07</v>
       </c>
       <c r="F147" t="inlineStr">
         <is>
@@ -4621,44 +4621,44 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Token-158</t>
+          <t>Token-160</t>
         </is>
       </c>
       <c r="B148" s="2" t="n">
-        <v>45663.50972222222</v>
+        <v>45663.5125</v>
       </c>
       <c r="C148" s="2" t="n">
-        <v>45698.30635824329</v>
+        <v>45698.29208832762</v>
       </c>
       <c r="D148" t="n">
-        <v>50107.16</v>
+        <v>50082.61</v>
       </c>
       <c r="E148" t="n">
-        <v>50093.66</v>
+        <v>46079.35</v>
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Inclusive Path 3 -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Token-159</t>
+          <t>Token-161</t>
         </is>
       </c>
       <c r="B149" s="2" t="n">
-        <v>45663.51111111111</v>
+        <v>45663.51388888889</v>
       </c>
       <c r="C149" s="2" t="n">
-        <v>45698.30982634045</v>
+        <v>45698.29562519141</v>
       </c>
       <c r="D149" t="n">
-        <v>50110.15</v>
+        <v>50085.7</v>
       </c>
       <c r="E149" t="n">
-        <v>50097.07</v>
+        <v>50073.07</v>
       </c>
       <c r="F149" t="inlineStr">
         <is>
@@ -4669,92 +4669,92 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Token-160</t>
+          <t>Token-162</t>
         </is>
       </c>
       <c r="B150" s="2" t="n">
-        <v>45663.5125</v>
+        <v>45663.51527777778</v>
       </c>
       <c r="C150" s="2" t="n">
-        <v>45698.42012668531</v>
+        <v>45698.29829485335</v>
       </c>
       <c r="D150" t="n">
-        <v>50266.98</v>
+        <v>50087.54</v>
       </c>
       <c r="E150" t="n">
-        <v>50099.52</v>
+        <v>50074.56</v>
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Inclusive Path 3 -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Token-161</t>
+          <t>Token-163</t>
         </is>
       </c>
       <c r="B151" s="2" t="n">
-        <v>45663.51388888889</v>
+        <v>45663.51666666667</v>
       </c>
       <c r="C151" s="2" t="n">
-        <v>45698.42366354911</v>
+        <v>45698.39916140353</v>
       </c>
       <c r="D151" t="n">
-        <v>50270.08</v>
+        <v>50230.79</v>
       </c>
       <c r="E151" t="n">
-        <v>50254.85</v>
+        <v>50077.84</v>
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Inclusive Path 3 -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Token-163</t>
+          <t>Token-164</t>
         </is>
       </c>
       <c r="B152" s="2" t="n">
-        <v>45663.51666666667</v>
+        <v>45663.51805555556</v>
       </c>
       <c r="C152" s="2" t="n">
-        <v>45699.29247073145</v>
+        <v>45698.40248701986</v>
       </c>
       <c r="D152" t="n">
-        <v>51517.16</v>
+        <v>50233.58</v>
       </c>
       <c r="E152" t="n">
-        <v>50342.03</v>
+        <v>50218.82</v>
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Inclusive Path 3 -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Token-164</t>
+          <t>Token-165</t>
         </is>
       </c>
       <c r="B153" s="2" t="n">
-        <v>45663.51805555556</v>
+        <v>45663.51944444444</v>
       </c>
       <c r="C153" s="2" t="n">
-        <v>45699.29629451008</v>
+        <v>45698.40700292798</v>
       </c>
       <c r="D153" t="n">
-        <v>51520.66</v>
+        <v>50238.08</v>
       </c>
       <c r="E153" t="n">
-        <v>51504.94</v>
+        <v>50222.08</v>
       </c>
       <c r="F153" t="inlineStr">
         <is>
@@ -4765,20 +4765,20 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Token-165</t>
+          <t>Token-166</t>
         </is>
       </c>
       <c r="B154" s="2" t="n">
-        <v>45663.51944444444</v>
+        <v>45663.52083333334</v>
       </c>
       <c r="C154" s="2" t="n">
-        <v>45699.30059781742</v>
+        <v>45698.41161148025</v>
       </c>
       <c r="D154" t="n">
-        <v>51524.86</v>
+        <v>50242.72</v>
       </c>
       <c r="E154" t="n">
-        <v>51510.46</v>
+        <v>50229.72</v>
       </c>
       <c r="F154" t="inlineStr">
         <is>
@@ -4789,44 +4789,44 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Token-166</t>
+          <t>Token-167</t>
         </is>
       </c>
       <c r="B155" s="2" t="n">
-        <v>45663.52083333334</v>
+        <v>45663.52222222222</v>
       </c>
       <c r="C155" s="2" t="n">
-        <v>45699.30411706315</v>
+        <v>45698.48173513204</v>
       </c>
       <c r="D155" t="n">
-        <v>51527.93</v>
+        <v>50341.7</v>
       </c>
       <c r="E155" t="n">
-        <v>51516.24</v>
+        <v>50234.44</v>
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Inclusive Path 3 -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>Token-167</t>
+          <t>Token-169</t>
         </is>
       </c>
       <c r="B156" s="2" t="n">
-        <v>45663.52222222222</v>
+        <v>45663.525</v>
       </c>
       <c r="C156" s="2" t="n">
-        <v>45699.30819924467</v>
+        <v>45699.29585030305</v>
       </c>
       <c r="D156" t="n">
-        <v>51531.81</v>
+        <v>51510.02</v>
       </c>
       <c r="E156" t="n">
-        <v>51517.19</v>
+        <v>51495.84</v>
       </c>
       <c r="F156" t="inlineStr">
         <is>
@@ -4837,20 +4837,20 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>Token-168</t>
+          <t>Token-170</t>
         </is>
       </c>
       <c r="B157" s="2" t="n">
-        <v>45663.52361111111</v>
+        <v>45663.52638888889</v>
       </c>
       <c r="C157" s="2" t="n">
-        <v>45699.31096786792</v>
+        <v>45699.29983493588</v>
       </c>
       <c r="D157" t="n">
-        <v>51533.79</v>
+        <v>51513.76</v>
       </c>
       <c r="E157" t="n">
-        <v>51520.77</v>
+        <v>51501.95</v>
       </c>
       <c r="F157" t="inlineStr">
         <is>
@@ -4861,20 +4861,20 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>Token-169</t>
+          <t>Token-171</t>
         </is>
       </c>
       <c r="B158" s="2" t="n">
-        <v>45663.525</v>
+        <v>45663.52777777778</v>
       </c>
       <c r="C158" s="2" t="n">
-        <v>45699.3139092267</v>
+        <v>45699.30441935965</v>
       </c>
       <c r="D158" t="n">
-        <v>51536.03</v>
+        <v>51518.36</v>
       </c>
       <c r="E158" t="n">
-        <v>51522.8</v>
+        <v>51504.01</v>
       </c>
       <c r="F158" t="inlineStr">
         <is>
@@ -4885,20 +4885,20 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>Token-170</t>
+          <t>Token-172</t>
         </is>
       </c>
       <c r="B159" s="2" t="n">
-        <v>45663.52638888889</v>
+        <v>45663.52916666667</v>
       </c>
       <c r="C159" s="2" t="n">
-        <v>45699.31851102235</v>
+        <v>45699.30761615394</v>
       </c>
       <c r="D159" t="n">
-        <v>51540.66</v>
+        <v>51520.97</v>
       </c>
       <c r="E159" t="n">
-        <v>51526.54</v>
+        <v>51508.04</v>
       </c>
       <c r="F159" t="inlineStr">
         <is>
@@ -4909,20 +4909,20 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>Token-171</t>
+          <t>Token-173</t>
         </is>
       </c>
       <c r="B160" s="2" t="n">
-        <v>45663.52777777778</v>
+        <v>45663.53055555555</v>
       </c>
       <c r="C160" s="2" t="n">
-        <v>45699.4213803859</v>
+        <v>45699.38435405059</v>
       </c>
       <c r="D160" t="n">
-        <v>51686.79</v>
+        <v>51629.47</v>
       </c>
       <c r="E160" t="n">
-        <v>51532.37</v>
+        <v>51509.5</v>
       </c>
       <c r="F160" t="inlineStr">
         <is>
@@ -4933,20 +4933,20 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>Token-173</t>
+          <t>Token-175</t>
         </is>
       </c>
       <c r="B161" s="2" t="n">
-        <v>45663.53055555555</v>
+        <v>45663.53333333333</v>
       </c>
       <c r="C161" s="2" t="n">
-        <v>45700.29231148768</v>
+        <v>45700.29233128639</v>
       </c>
       <c r="D161" t="n">
-        <v>52936.93</v>
+        <v>52932.96</v>
       </c>
       <c r="E161" t="n">
-        <v>51798.45</v>
+        <v>51756</v>
       </c>
       <c r="F161" t="inlineStr">
         <is>
@@ -4957,44 +4957,44 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>Token-174</t>
+          <t>Token-178</t>
         </is>
       </c>
       <c r="B162" s="2" t="n">
-        <v>45663.53194444445</v>
+        <v>45663.5375</v>
       </c>
       <c r="C162" s="2" t="n">
-        <v>45700.2951136826</v>
+        <v>45700.51325968159</v>
       </c>
       <c r="D162" t="n">
-        <v>52938.96</v>
+        <v>53245.09</v>
       </c>
       <c r="E162" t="n">
-        <v>48968.17</v>
+        <v>53131.53</v>
       </c>
       <c r="F162" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Inclusive Path 3 -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>Token-175</t>
+          <t>Token-179</t>
         </is>
       </c>
       <c r="B163" s="2" t="n">
-        <v>45663.53333333333</v>
+        <v>45663.53888888889</v>
       </c>
       <c r="C163" s="2" t="n">
-        <v>45700.29794719649</v>
+        <v>45700.5164313999</v>
       </c>
       <c r="D163" t="n">
-        <v>52941.04</v>
+        <v>53247.66</v>
       </c>
       <c r="E163" t="n">
-        <v>52927.66</v>
+        <v>53232.72</v>
       </c>
       <c r="F163" t="inlineStr">
         <is>
@@ -5005,20 +5005,20 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>Token-176</t>
+          <t>Token-180</t>
         </is>
       </c>
       <c r="B164" s="2" t="n">
-        <v>45663.53472222222</v>
+        <v>45663.54027777778</v>
       </c>
       <c r="C164" s="2" t="n">
-        <v>45700.30229236458</v>
+        <v>45700.51968190433</v>
       </c>
       <c r="D164" t="n">
-        <v>52945.3</v>
+        <v>53250.34</v>
       </c>
       <c r="E164" t="n">
-        <v>52929.96</v>
+        <v>53237.71</v>
       </c>
       <c r="F164" t="inlineStr">
         <is>
@@ -5029,20 +5029,20 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>Token-178</t>
+          <t>Token-183</t>
         </is>
       </c>
       <c r="B165" s="2" t="n">
-        <v>45663.5375</v>
+        <v>45664.29444444444</v>
       </c>
       <c r="C165" s="2" t="n">
-        <v>45700.3822421685</v>
+        <v>45701.40679131757</v>
       </c>
       <c r="D165" t="n">
-        <v>53056.43</v>
+        <v>53441.78</v>
       </c>
       <c r="E165" t="n">
-        <v>53041.01</v>
+        <v>53427.3</v>
       </c>
       <c r="F165" t="inlineStr">
         <is>
@@ -5053,44 +5053,44 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Token-179</t>
+          <t>Token-184</t>
         </is>
       </c>
       <c r="B166" s="2" t="n">
-        <v>45663.53888888889</v>
+        <v>45664.29583333333</v>
       </c>
       <c r="C166" s="2" t="n">
-        <v>45700.4827020833</v>
+        <v>45701.41071713808</v>
       </c>
       <c r="D166" t="n">
-        <v>53199.09</v>
+        <v>53445.43</v>
       </c>
       <c r="E166" t="n">
-        <v>53044.99</v>
+        <v>53434.21</v>
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Inclusive Path 3 -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Token-181</t>
+          <t>Token-185</t>
         </is>
       </c>
       <c r="B167" s="2" t="n">
-        <v>45664.29166666666</v>
+        <v>45664.29722222222</v>
       </c>
       <c r="C167" s="2" t="n">
-        <v>45701.29499762179</v>
+        <v>45701.41509144931</v>
       </c>
       <c r="D167" t="n">
-        <v>53284.8</v>
+        <v>53449.73</v>
       </c>
       <c r="E167" t="n">
-        <v>53271.42</v>
+        <v>53435.62</v>
       </c>
       <c r="F167" t="inlineStr">
         <is>
@@ -5101,20 +5101,20 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>Token-182</t>
+          <t>Token-186</t>
         </is>
       </c>
       <c r="B168" s="2" t="n">
-        <v>45664.29305555556</v>
+        <v>45664.29861111111</v>
       </c>
       <c r="C168" s="2" t="n">
-        <v>45701.29951676823</v>
+        <v>45701.41938441905</v>
       </c>
       <c r="D168" t="n">
-        <v>53289.3</v>
+        <v>53453.91</v>
       </c>
       <c r="E168" t="n">
-        <v>53273.29</v>
+        <v>53439.36</v>
       </c>
       <c r="F168" t="inlineStr">
         <is>
@@ -5125,20 +5125,20 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>Token-183</t>
+          <t>Token-187</t>
         </is>
       </c>
       <c r="B169" s="2" t="n">
-        <v>45664.29444444444</v>
+        <v>45664.3</v>
       </c>
       <c r="C169" s="2" t="n">
-        <v>45701.30268403094</v>
+        <v>45701.42392984097</v>
       </c>
       <c r="D169" t="n">
-        <v>53291.87</v>
+        <v>53458.46</v>
       </c>
       <c r="E169" t="n">
-        <v>53277.91</v>
+        <v>53444.54</v>
       </c>
       <c r="F169" t="inlineStr">
         <is>
@@ -5149,20 +5149,20 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>Token-184</t>
+          <t>Token-188</t>
         </is>
       </c>
       <c r="B170" s="2" t="n">
-        <v>45664.29583333333</v>
+        <v>45664.30138888889</v>
       </c>
       <c r="C170" s="2" t="n">
-        <v>45701.30726374243</v>
+        <v>45701.42722114671</v>
       </c>
       <c r="D170" t="n">
-        <v>53296.46</v>
+        <v>53461.2</v>
       </c>
       <c r="E170" t="n">
-        <v>53281.49</v>
+        <v>53450.44</v>
       </c>
       <c r="F170" t="inlineStr">
         <is>
@@ -5173,20 +5173,20 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>Token-185</t>
+          <t>Token-189</t>
         </is>
       </c>
       <c r="B171" s="2" t="n">
-        <v>45664.29722222222</v>
+        <v>45664.30277777778</v>
       </c>
       <c r="C171" s="2" t="n">
-        <v>45701.31117753976</v>
+        <v>45701.43152911676</v>
       </c>
       <c r="D171" t="n">
-        <v>53300.1</v>
+        <v>53465.4</v>
       </c>
       <c r="E171" t="n">
-        <v>53286.09</v>
+        <v>53450.47</v>
       </c>
       <c r="F171" t="inlineStr">
         <is>
@@ -5197,20 +5197,20 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>Token-186</t>
+          <t>Token-190</t>
         </is>
       </c>
       <c r="B172" s="2" t="n">
-        <v>45664.29861111111</v>
+        <v>45664.30416666667</v>
       </c>
       <c r="C172" s="2" t="n">
-        <v>45701.31558700051</v>
+        <v>45701.43457915749</v>
       </c>
       <c r="D172" t="n">
-        <v>53304.45</v>
+        <v>53467.79</v>
       </c>
       <c r="E172" t="n">
-        <v>53290.36</v>
+        <v>53455.18</v>
       </c>
       <c r="F172" t="inlineStr">
         <is>
@@ -5221,20 +5221,20 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>Token-187</t>
+          <t>Token-191</t>
         </is>
       </c>
       <c r="B173" s="2" t="n">
-        <v>45664.3</v>
+        <v>45664.30555555555</v>
       </c>
       <c r="C173" s="2" t="n">
-        <v>45701.3187483165</v>
+        <v>45701.43800120219</v>
       </c>
       <c r="D173" t="n">
-        <v>53307</v>
+        <v>53470.72</v>
       </c>
       <c r="E173" t="n">
-        <v>53294.06</v>
+        <v>53456.85</v>
       </c>
       <c r="F173" t="inlineStr">
         <is>
@@ -5245,20 +5245,20 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>Token-188</t>
+          <t>Token-192</t>
         </is>
       </c>
       <c r="B174" s="2" t="n">
-        <v>45664.30138888889</v>
+        <v>45664.30694444444</v>
       </c>
       <c r="C174" s="2" t="n">
-        <v>45701.32328214369</v>
+        <v>45701.44262634122</v>
       </c>
       <c r="D174" t="n">
-        <v>53311.53</v>
+        <v>53475.38</v>
       </c>
       <c r="E174" t="n">
-        <v>53296.5</v>
+        <v>53462.67</v>
       </c>
       <c r="F174" t="inlineStr">
         <is>
@@ -5269,20 +5269,20 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>Token-189</t>
+          <t>Token-193</t>
         </is>
       </c>
       <c r="B175" s="2" t="n">
-        <v>45664.30277777778</v>
+        <v>45664.30833333333</v>
       </c>
       <c r="C175" s="2" t="n">
-        <v>45701.32769808429</v>
+        <v>45701.44712847074</v>
       </c>
       <c r="D175" t="n">
-        <v>53315.89</v>
+        <v>53479.86</v>
       </c>
       <c r="E175" t="n">
-        <v>53301.97</v>
+        <v>53464.03</v>
       </c>
       <c r="F175" t="inlineStr">
         <is>
@@ -5293,20 +5293,20 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>Token-190</t>
+          <t>Token-194</t>
         </is>
       </c>
       <c r="B176" s="2" t="n">
-        <v>45664.30416666667</v>
+        <v>45664.30972222222</v>
       </c>
       <c r="C176" s="2" t="n">
-        <v>45701.33200106426</v>
+        <v>45701.4509953435</v>
       </c>
       <c r="D176" t="n">
-        <v>53320.08</v>
+        <v>53483.43</v>
       </c>
       <c r="E176" t="n">
-        <v>53304.94</v>
+        <v>53468.9</v>
       </c>
       <c r="F176" t="inlineStr">
         <is>
@@ -5317,44 +5317,44 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>Token-192</t>
+          <t>Token-195</t>
         </is>
       </c>
       <c r="B177" s="2" t="n">
-        <v>45664.30694444444</v>
+        <v>45664.31111111111</v>
       </c>
       <c r="C177" s="2" t="n">
-        <v>45701.40246767899</v>
+        <v>45702.29250352156</v>
       </c>
       <c r="D177" t="n">
-        <v>53417.55</v>
+        <v>54693.21</v>
       </c>
       <c r="E177" t="n">
-        <v>53403.37</v>
+        <v>53473.67</v>
       </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Inclusive Path 3 -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>Token-193</t>
+          <t>Token-196</t>
         </is>
       </c>
       <c r="B178" s="2" t="n">
-        <v>45664.30833333333</v>
+        <v>45664.3125</v>
       </c>
       <c r="C178" s="2" t="n">
-        <v>45701.4063934995</v>
+        <v>45702.29522832121</v>
       </c>
       <c r="D178" t="n">
-        <v>53421.21</v>
+        <v>54695.13</v>
       </c>
       <c r="E178" t="n">
-        <v>53410.16</v>
+        <v>54680.46</v>
       </c>
       <c r="F178" t="inlineStr">
         <is>
@@ -5365,20 +5365,20 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>Token-195</t>
+          <t>Token-199</t>
         </is>
       </c>
       <c r="B179" s="2" t="n">
-        <v>45664.31111111111</v>
+        <v>45664.31666666667</v>
       </c>
       <c r="C179" s="2" t="n">
-        <v>45701.51598413756</v>
+        <v>45702.46139628292</v>
       </c>
       <c r="D179" t="n">
-        <v>53575.02</v>
+        <v>54928.41</v>
       </c>
       <c r="E179" t="n">
-        <v>53562.17</v>
+        <v>54913.42</v>
       </c>
       <c r="F179" t="inlineStr">
         <is>
@@ -5389,20 +5389,20 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>Token-196</t>
+          <t>Token-200</t>
         </is>
       </c>
       <c r="B180" s="2" t="n">
-        <v>45664.3125</v>
+        <v>45664.31805555556</v>
       </c>
       <c r="C180" s="2" t="n">
-        <v>45701.51903417829</v>
+        <v>45702.46437282553</v>
       </c>
       <c r="D180" t="n">
-        <v>53577.41</v>
+        <v>54930.7</v>
       </c>
       <c r="E180" t="n">
-        <v>53563.76</v>
+        <v>54917.54</v>
       </c>
       <c r="F180" t="inlineStr">
         <is>
@@ -5413,20 +5413,20 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>Token-197</t>
+          <t>Token-201</t>
         </is>
       </c>
       <c r="B181" s="2" t="n">
-        <v>45664.31388888889</v>
+        <v>45664.31944444445</v>
       </c>
       <c r="C181" s="2" t="n">
-        <v>45701.52245622299</v>
+        <v>45702.46790968873</v>
       </c>
       <c r="D181" t="n">
-        <v>53580.34</v>
+        <v>54933.79</v>
       </c>
       <c r="E181" t="n">
-        <v>53567.9</v>
+        <v>54919.42</v>
       </c>
       <c r="F181" t="inlineStr">
         <is>
@@ -5437,44 +5437,44 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>Token-198</t>
+          <t>Token-204</t>
         </is>
       </c>
       <c r="B182" s="2" t="n">
-        <v>45664.31527777778</v>
+        <v>45664.32361111111</v>
       </c>
       <c r="C182" s="2" t="n">
-        <v>45701.52708136202</v>
+        <v>45705.40320214732</v>
       </c>
       <c r="D182" t="n">
-        <v>53585</v>
+        <v>59154.61</v>
       </c>
       <c r="E182" t="n">
-        <v>53568.92</v>
+        <v>59076.66</v>
       </c>
       <c r="F182" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Inclusive Path 3 -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>Token-200</t>
+          <t>Token-205</t>
         </is>
       </c>
       <c r="B183" s="2" t="n">
-        <v>45664.31805555556</v>
+        <v>45664.325</v>
       </c>
       <c r="C183" s="2" t="n">
-        <v>45702.29553353944</v>
+        <v>45705.4067839331</v>
       </c>
       <c r="D183" t="n">
-        <v>54687.57</v>
+        <v>59157.77</v>
       </c>
       <c r="E183" t="n">
-        <v>54673.35</v>
+        <v>59141.97</v>
       </c>
       <c r="F183" t="inlineStr">
         <is>
@@ -5485,20 +5485,20 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>Token-201</t>
+          <t>Token-206</t>
         </is>
       </c>
       <c r="B184" s="2" t="n">
-        <v>45664.31944444445</v>
+        <v>45664.32638888889</v>
       </c>
       <c r="C184" s="2" t="n">
-        <v>45702.29917455961</v>
+        <v>45705.4111048554</v>
       </c>
       <c r="D184" t="n">
-        <v>54690.81</v>
+        <v>59161.99</v>
       </c>
       <c r="E184" t="n">
-        <v>54676.95</v>
+        <v>59149.35</v>
       </c>
       <c r="F184" t="inlineStr">
         <is>
@@ -5509,20 +5509,20 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>Token-202</t>
+          <t>Token-207</t>
         </is>
       </c>
       <c r="B185" s="2" t="n">
-        <v>45664.32083333333</v>
+        <v>45664.32777777778</v>
       </c>
       <c r="C185" s="2" t="n">
-        <v>45702.30283842242</v>
+        <v>45705.41461967911</v>
       </c>
       <c r="D185" t="n">
-        <v>54694.09</v>
+        <v>59165.05</v>
       </c>
       <c r="E185" t="n">
-        <v>54681.23</v>
+        <v>59152.16</v>
       </c>
       <c r="F185" t="inlineStr">
         <is>
@@ -5533,68 +5533,68 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>Token-203</t>
+          <t>Token-208</t>
         </is>
       </c>
       <c r="B186" s="2" t="n">
-        <v>45664.32222222222</v>
+        <v>45664.32916666667</v>
       </c>
       <c r="C186" s="2" t="n">
-        <v>45702.3075126483</v>
+        <v>45705.52117415984</v>
       </c>
       <c r="D186" t="n">
-        <v>54698.82</v>
+        <v>59316.49</v>
       </c>
       <c r="E186" t="n">
-        <v>54682.84</v>
+        <v>59154.28</v>
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Inclusive Path 3 -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>Token-18</t>
+          <t>Token-209</t>
         </is>
       </c>
       <c r="B187" s="2" t="n">
-        <v>45663.31527777778</v>
+        <v>45664.33055555556</v>
       </c>
       <c r="C187" s="2" t="n">
-        <v>45702.36922619887</v>
+        <v>45706.29217860114</v>
       </c>
       <c r="D187" t="n">
-        <v>56237.69</v>
+        <v>60424.74</v>
       </c>
       <c r="E187" t="n">
-        <v>55056.17</v>
+        <v>59304.24</v>
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Inclusive Path 3 -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>Token-205</t>
+          <t>Token-210</t>
         </is>
       </c>
       <c r="B188" s="2" t="n">
-        <v>45664.325</v>
+        <v>45664.33194444444</v>
       </c>
       <c r="C188" s="2" t="n">
-        <v>45702.37353985205</v>
+        <v>45706.29523010387</v>
       </c>
       <c r="D188" t="n">
-        <v>54789.9</v>
+        <v>60427.13</v>
       </c>
       <c r="E188" t="n">
-        <v>54774.55</v>
+        <v>60414.8</v>
       </c>
       <c r="F188" t="inlineStr">
         <is>
@@ -5605,20 +5605,20 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>Token-206</t>
+          <t>Token-211</t>
         </is>
       </c>
       <c r="B189" s="2" t="n">
-        <v>45664.32638888889</v>
+        <v>45664.33333333334</v>
       </c>
       <c r="C189" s="2" t="n">
-        <v>45702.37805717561</v>
+        <v>45706.29977820549</v>
       </c>
       <c r="D189" t="n">
-        <v>54794.4</v>
+        <v>60431.68</v>
       </c>
       <c r="E189" t="n">
-        <v>54781.48</v>
+        <v>60418.03</v>
       </c>
       <c r="F189" t="inlineStr">
         <is>
@@ -5629,20 +5629,20 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>Token-207</t>
+          <t>Token-212</t>
         </is>
       </c>
       <c r="B190" s="2" t="n">
-        <v>45664.32777777778</v>
+        <v>45664.33472222222</v>
       </c>
       <c r="C190" s="2" t="n">
-        <v>45702.38195778054</v>
+        <v>45706.30373744204</v>
       </c>
       <c r="D190" t="n">
-        <v>54798.02</v>
+        <v>60435.38</v>
       </c>
       <c r="E190" t="n">
-        <v>54784.57</v>
+        <v>60423.35</v>
       </c>
       <c r="F190" t="inlineStr">
         <is>
@@ -5653,142 +5653,22 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>Token-208</t>
+          <t>Token-213</t>
         </is>
       </c>
       <c r="B191" s="2" t="n">
-        <v>45664.32916666667</v>
+        <v>45664.33611111111</v>
       </c>
       <c r="C191" s="2" t="n">
-        <v>45702.47611596811</v>
+        <v>45706.30830026272</v>
       </c>
       <c r="D191" t="n">
-        <v>54931.61</v>
+        <v>60439.95</v>
       </c>
       <c r="E191" t="n">
-        <v>54787.25</v>
+        <v>60424.63</v>
       </c>
       <c r="F191" t="inlineStr">
-        <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Inclusive Path 3 -&gt; Unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="192">
-      <c r="A192" t="inlineStr">
-        <is>
-          <t>Token-209</t>
-        </is>
-      </c>
-      <c r="B192" s="2" t="n">
-        <v>45664.33055555556</v>
-      </c>
-      <c r="C192" s="2" t="n">
-        <v>45702.52775644851</v>
-      </c>
-      <c r="D192" t="n">
-        <v>55003.97</v>
-      </c>
-      <c r="E192" t="n">
-        <v>54919.65</v>
-      </c>
-      <c r="F192" t="inlineStr">
-        <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Inclusive Path 3 -&gt; Unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="193">
-      <c r="A193" t="inlineStr">
-        <is>
-          <t>Token-210</t>
-        </is>
-      </c>
-      <c r="B193" s="2" t="n">
-        <v>45664.33194444444</v>
-      </c>
-      <c r="C193" s="2" t="n">
-        <v>45702.53118237798</v>
-      </c>
-      <c r="D193" t="n">
-        <v>55006.9</v>
-      </c>
-      <c r="E193" t="n">
-        <v>54993.57</v>
-      </c>
-      <c r="F193" t="inlineStr">
-        <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="194">
-      <c r="A194" t="inlineStr">
-        <is>
-          <t>Token-211</t>
-        </is>
-      </c>
-      <c r="B194" s="2" t="n">
-        <v>45664.33333333334</v>
-      </c>
-      <c r="C194" s="2" t="n">
-        <v>45702.53501894678</v>
-      </c>
-      <c r="D194" t="n">
-        <v>55010.43</v>
-      </c>
-      <c r="E194" t="n">
-        <v>54997.8</v>
-      </c>
-      <c r="F194" t="inlineStr">
-        <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="195">
-      <c r="A195" t="inlineStr">
-        <is>
-          <t>Token-212</t>
-        </is>
-      </c>
-      <c r="B195" s="2" t="n">
-        <v>45664.33472222222</v>
-      </c>
-      <c r="C195" s="2" t="n">
-        <v>45702.53823357952</v>
-      </c>
-      <c r="D195" t="n">
-        <v>55013.06</v>
-      </c>
-      <c r="E195" t="n">
-        <v>55002.1</v>
-      </c>
-      <c r="F195" t="inlineStr">
-        <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="196">
-      <c r="A196" t="inlineStr">
-        <is>
-          <t>Token-213</t>
-        </is>
-      </c>
-      <c r="B196" s="2" t="n">
-        <v>45664.33611111111</v>
-      </c>
-      <c r="C196" s="2" t="n">
-        <v>45705.29166666666</v>
-      </c>
-      <c r="D196" t="n">
-        <v>58976</v>
-      </c>
-      <c r="E196" t="n">
-        <v>55002.3</v>
-      </c>
-      <c r="F196" t="inlineStr">
         <is>
           <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
@@ -5837,7 +5717,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="4">
@@ -5857,7 +5737,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>35610.18</v>
+        <v>35095.94</v>
       </c>
     </row>
     <row r="6">
@@ -5867,7 +5747,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>53378.56</v>
+        <v>53468.09</v>
       </c>
     </row>
     <row r="7">
@@ -5877,7 +5757,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>35402.82</v>
+        <v>34925.89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
simulation_engine re-engineered using CHATGPT but does not yet run.  Previous simulation_engine_old is from claude sonnet and the simulation was not progressing beyond the first activity
</commit_message>
<xml_diff>
--- a/5.5.13 Real Property-Monthly Reviews-Inclusive_results.xlsx
+++ b/5.5.13 Real Property-Monthly Reviews-Inclusive_results.xlsx
@@ -7,41 +7,16 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Completed Tokens" sheetId="1" r:id="rId1"/>
-    <sheet name="Activity Statistics" sheetId="2" r:id="rId2"/>
-    <sheet name="Resource Utilization" sheetId="3" r:id="rId3"/>
-    <sheet name="Simulation Parameters" sheetId="4" r:id="rId4"/>
+    <sheet name="Activity Statistics" sheetId="1" r:id="rId1"/>
+    <sheet name="Resource Utilization" sheetId="2" r:id="rId2"/>
+    <sheet name="Simulation Parameters" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
-  <si>
-    <t>Token ID</t>
-  </si>
-  <si>
-    <t>Start Time</t>
-  </si>
-  <si>
-    <t>End Time</t>
-  </si>
-  <si>
-    <t>Total Duration (min)</t>
-  </si>
-  <si>
-    <t>Wait Time (min)</t>
-  </si>
-  <si>
-    <t>Path</t>
-  </si>
-  <si>
-    <t>Token-1</t>
-  </si>
-  <si>
-    <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Unknown</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>Activity</t>
   </si>
@@ -67,18 +42,6 @@
     <t>Review AM using Asset Change Tracker (5.5.13.1)</t>
   </si>
   <si>
-    <t>Complete /Accurate?</t>
-  </si>
-  <si>
-    <t>Note Accuracy in Asset Change Tracker (5.5.13.2)</t>
-  </si>
-  <si>
-    <t>Work with REO RPO to Correct (5.5.13.3)</t>
-  </si>
-  <si>
-    <t>Unknown</t>
-  </si>
-  <si>
     <t>Resource</t>
   </si>
   <si>
@@ -113,18 +76,12 @@
   </si>
   <si>
     <t>Max Interval (min)</t>
-  </si>
-  <si>
-    <t>Average Process Time (min)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
-  </numFmts>
   <fonts count="2">
     <font>
       <sz val="11"/>
@@ -177,12 +134,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -477,7 +433,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -504,20 +460,40 @@
       <c r="A2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="2">
-        <v>45726.33333333334</v>
-      </c>
-      <c r="C2" s="2">
-        <v>45726.34843493204</v>
+      <c r="B2">
+        <v>227</v>
+      </c>
+      <c r="C2">
+        <v>227</v>
       </c>
       <c r="D2">
-        <v>21.75</v>
+        <v>0</v>
       </c>
       <c r="E2">
-        <v>7.17</v>
-      </c>
-      <c r="F2" t="s">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" t="s">
         <v>7</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>10.5</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>10.5</v>
       </c>
     </row>
   </sheetData>
@@ -527,147 +503,23 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
         <v>10</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" t="s">
-        <v>14</v>
-      </c>
       <c r="B2">
-        <v>500</v>
-      </c>
-      <c r="C2">
-        <v>500</v>
-      </c>
-      <c r="D2">
-        <v>0</v>
-      </c>
-      <c r="E2">
-        <v>0</v>
-      </c>
-      <c r="F2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
-      <c r="A3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="C3">
-        <v>2</v>
-      </c>
-      <c r="D3">
-        <v>7.93</v>
-      </c>
-      <c r="E3">
-        <v>3.84</v>
-      </c>
-      <c r="F3">
-        <v>11.77</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
-      <c r="A4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4">
-        <v>2</v>
-      </c>
-      <c r="C4">
-        <v>2</v>
-      </c>
-      <c r="D4">
-        <v>0</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-      <c r="F4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
-      <c r="A5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5">
-        <v>1</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5">
-        <v>5.89</v>
-      </c>
-      <c r="E5">
-        <v>7.17</v>
-      </c>
-      <c r="F5">
-        <v>13.06</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
-      <c r="A6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B6">
-        <v>1</v>
-      </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-      <c r="D6">
-        <v>159.23</v>
-      </c>
-      <c r="E6">
-        <v>0</v>
-      </c>
-      <c r="F6">
-        <v>159.23</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
-      <c r="A7" t="s">
-        <v>19</v>
-      </c>
-      <c r="B7">
-        <v>1</v>
-      </c>
-      <c r="C7">
-        <v>1</v>
-      </c>
-      <c r="D7">
-        <v>0</v>
-      </c>
-      <c r="E7">
-        <v>0</v>
-      </c>
-      <c r="F7">
-        <v>0</v>
+        <v>0.1458096456018518</v>
       </c>
     </row>
   </sheetData>
@@ -677,78 +529,52 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="B2">
-        <v>0.0050338662345679</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B2">
-        <v>500</v>
+        <v>227</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="B4">
-        <v>300</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="B5">
-        <v>500</v>
+        <v>300</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="B6">
         <v>4</v>
@@ -756,7 +582,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="B7">
         <v>5</v>
@@ -764,18 +590,10 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="B8">
         <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2">
-      <c r="A9" t="s">
-        <v>32</v>
-      </c>
-      <c r="B9">
-        <v>21.75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>